<commit_message>
Edit BCIO_External_Imports.xlsx: update 1, add 1
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -678,7 +678,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>environment [ENVO:01000254]; research facility [ENVO:00000469]; park [ENVO:00000562]; forest [ENVO:00000111]; beach [ENVO:00000091]; grassland [ENVO:00000106]; road [ENVO:00000064];﻿ecosystem [ENVO:01001110];﻿environmental disposition [ENVO:01000452]; environmental system [ENVO:01000254]</t>
+          <t>environment [ENVO:01000254]; research facility [ENVO:00000469]; forest [ENVO:00000111]; beach [ENVO:00000091]; grassland [ENVO:00000106]; road [ENVO:00000064];﻿ecosystem [ENVO:01001110];﻿environmental disposition [ENVO:01000452]; environmental system [ENVO:01000254]</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1145,6 +1145,36 @@
           <t>all</t>
         </is>
       </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ENVO</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/envo.owl</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/envo/releases/2025-02-05/envo.owl</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>anthropogenic geographic feature [ENVO:00000002]</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">park [ENVO:00000562]; </t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update ROOT_ID of Row 21 in BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -1164,7 +1164,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>anthropogenic geographic feature [ENVO:00000002]</t>
+          <t xml:space="preserve">park [ENVO:00000562]; </t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1172,9 +1172,6 @@
           <t xml:space="preserve">park [ENVO:00000562]; </t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2 terms in BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -678,12 +678,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>environment [ENVO:01000254]; research facility [ENVO:00000469]; forest [ENVO:00000111]; beach [ENVO:00000091]; grassland [ENVO:00000106]; road [ENVO:00000064];﻿ecosystem [ENVO:01001110];﻿environmental disposition [ENVO:01000452]; environmental system [ENVO:01000254]</t>
+          <t>environment [ENVO:01000254]; research facility [ENVO:00000469];ecosystem [ENVO:01001110];﻿environmental disposition [ENVO:01000452]; environmental system [ENVO:01000254]</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>facility [ENVO:03501288]</t>
+          <t xml:space="preserve">facility [ENVO:03501288]; </t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1164,12 +1164,18 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">park [ENVO:00000562]; </t>
+          <t>entity [BFO:0000001]</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">park [ENVO:00000562]; </t>
+          <t xml:space="preserve">park [ENVO:00000562]; road [ENVO:00000064];﻿ beach [ENVO:00000091]; forest [ENVO:00000111];  grassland [ENVO:00000106]; </t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit BCIO_External_Imports.xlsx: update 2, delete 2
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -609,17 +609,18 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>realizable entity [BFO:0000017]</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">patient role [OBI:0000093]; plan [OBI:0000260]; </t>
-        </is>
-      </c>
+          <t xml:space="preserve">patient role [OBI:0000093]; plan [OBI:0000260]; organisation [OBI:0000245]; </t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>none</t>
         </is>
       </c>
     </row>
@@ -678,12 +679,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>environment [ENVO:01000254]; research facility [ENVO:00000469];ecosystem [ENVO:01001110];﻿environmental disposition [ENVO:01000452]; environmental system [ENVO:01000254]</t>
+          <t xml:space="preserve">environment [ENVO:01000254]; research facility [ENVO:00000469];ecosystem [ENVO:01001110];﻿environmental disposition [ENVO:01000452]; environmental system [ENVO:01000254]; park [ENVO:00000562]; road [ENVO:00000064];﻿ beach [ENVO:00000091]; forest [ENVO:00000111];  grassland [ENVO:00000106]; </t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">facility [ENVO:03501288]; </t>
+          <t>anthropogenic geographic feature [ENVO:00000002]; geographic feature [ENVO:00000000]; astronomical body part [ENVO:01000813]; woodland area [ENVO:00000109]; vegetated area [ENVO:01001305]; terrestrial environmental zone [ENVO:01001199]; terrestrial biome [ENVO:00000446]; biome [ENVO:00000428]; biosphere [ENVO:01000817];  shore [ENVO:00000304]; surface landform [ENVO:01001884]; landform [ENVO:01001886]; solid astronomical body part [ENVO:00000191]; compound astronomical body part [ENVO:01001784]; constructed pavement [ENVO:01001272]; transport feature [ENVO:00000010]; human construction [ENVO:00000070]; construction [ENVO:01001813]; land [ENVO:01001785]; terrestrial ecosystem [ENVO:01001790];  solid surface layer [ENVO:01001311]; surface layer [ENVO:00010504]; layer [ENVO:01000281]; interface layer [http://purl.obolibrary.org/obo/ENVO_01001684]</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1111,70 +1112,6 @@
       <c r="G21" t="inlineStr">
         <is>
           <t>all</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>OBI</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/obi.owl</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/obi/2025-01-09/obi.owl</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>material entity [BFO:0000040]</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">organisation [OBI:0000245]; </t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ENVO</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/envo.owl</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/envo/releases/2025-02-05/envo.owl</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>entity [BFO:0000001]</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">park [ENVO:00000562]; road [ENVO:00000064];﻿ beach [ENVO:00000091]; forest [ENVO:00000111];  grassland [ENVO:00000106]; </t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>none</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Delete Row 17 from BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1021,17 +1021,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SDGIO</t>
+          <t>OPMI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/SDG-InterfaceOntology/sdgio/master/sdgio.owl</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/SDG-InterfaceOntology/sdgio/d6f94a02435d103c6fe6fce057fbbe43d33f94aa/sdgio.owl</t>
+          <t>http://purl.obolibrary.org/obo/opmi.owl</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1041,74 +1036,42 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>owner [SDGIO:00010028]; employment status [SDGIO:00010029]; education process [SDGIO:00010001]; unemployed status [SDGIO:00010026]</t>
+          <t>socioeconomic status [OPMI:0000121]</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>all</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>"SDGIO: http://purl.unep.org/sdg/SDGIO_"</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OPMI</t>
+          <t>COB</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/opmi.owl</t>
+          <t>http://purl.obolibrary.org/obo/COB.owl</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/OBOFoundry/COB/2b7d820f804fc9fa17aba5a21a9ce2f821dc5c83/cob.owl</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>entity [BFO:0000001]</t>
+          <t>process [BFO:0000015]</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>socioeconomic status [OPMI:0000121]</t>
+          <t>planned process [COB:0000082]</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>COB</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/COB.owl</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/OBOFoundry/COB/2b7d820f804fc9fa17aba5a21a9ce2f821dc5c83/cob.owl</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>process [BFO:0000015]</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>planned process [COB:0000082]</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
         <is>
           <t>all</t>
         </is>

</xml_diff>

<commit_message>
Update Row 5 in BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -639,19 +639,15 @@
           <t>http://purl.obolibrary.org/obo/sepio/releases/2023-06-13/sepio.owl</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>research activity [SEPIO:0000004]</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">research study [SEPIO:0000125] </t>
+          <t>research study [SEPIO:0000125] ; research activity [SEPIO:0000004]</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>none</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ROOT_ID of Row 5 in BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -639,7 +639,11 @@
           <t>http://purl.obolibrary.org/obo/sepio/releases/2023-06-13/sepio.owl</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>entity [BFO:0000001]</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>research study [SEPIO:0000125] ; research activity [SEPIO:0000004]</t>

</xml_diff>